<commit_message>
chore: add updated pipe size Excel files and seed script
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/PIPES SIZE MASTER CS & AS PIPES.xlsx
+++ b/documents/PIPES SIZE MASTER CS & AS PIPES.xlsx
@@ -38,580 +38,580 @@
 (kg/m)</t>
   </si>
   <si>
-    <t>1/2" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>1/2" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>3/4" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>1" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>1" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>1" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>1" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>1" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>1" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>1" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>1.25" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>1.5" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>2" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>2" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>2" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>2" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>2" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>2" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>2" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>2.5" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>3" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>3" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>3" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>3" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>3" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>3" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>3" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>4" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>4" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>4" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>4" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>4" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>4" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>4" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>4" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>5" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>5" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>5" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>5" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>5" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>5" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>5" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>5" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>6" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>6" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>6" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>6" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>6" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>6" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>6" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>6" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>8" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>8" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>8" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>8" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>10" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>10" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>10" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>10" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>12" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>12" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>12" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>12" NB X Sch XXS</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>14" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>14" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>14" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>16" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>16" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>16" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>18" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>18" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>18" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>20" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>20" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>20" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>22" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>22" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>22" NB X Sch 160</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 10</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 20</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 30</t>
-  </si>
-  <si>
-    <t>24" NB X Sch STD</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 40</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 60</t>
-  </si>
-  <si>
-    <t>24" NB X Sch XS</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 80</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 100</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 120</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 140</t>
-  </si>
-  <si>
-    <t>24" NB X Sch 160</t>
-  </si>
-  <si>
     <t>Size</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>1/2"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>3/4"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>1"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>1"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>1"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>1"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>1"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>1"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>1"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>1.25"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>1.5"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>2"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>2"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>2"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>2"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>2"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>2"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>2"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>2.5"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>3"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>3"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>3"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>3"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>3"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>3"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>3"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>4"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>4"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>4"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>4"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>4"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>4"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>4"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>4"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>5"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>5"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>5"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>5"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>5"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>5"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>5"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>5"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>6"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>6"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>6"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>6"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>6"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>6"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>6"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>6"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>8"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>8"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>8"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>8"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>10"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>10"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>10"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>10"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>12"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>12"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>12"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>12"NB X SCH XXS</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>14"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>14"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>14"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>16"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>16"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>16"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>18"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>18"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>18"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>20"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>20"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>20"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>22"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>22"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>22"NB X SCH 160</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 10</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 20</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 30</t>
+  </si>
+  <si>
+    <t>24"NB X SCH STD</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 40</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 60</t>
+  </si>
+  <si>
+    <t>24"NB X SCH XS</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 80</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 100</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 120</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 140</t>
+  </si>
+  <si>
+    <t>24"NB X SCH 160</t>
   </si>
 </sst>
 </file>
@@ -983,7 +983,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>194</v>
+        <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="3">
         <v>21.3</v>
@@ -1006,13 +1006,13 @@
         <v>2.11</v>
       </c>
       <c r="D2" s="4">
-        <f>SUM(B2-C2)*C2*0.0246615</f>
+        <f t="shared" ref="D2:D33" si="0">SUM(B2-C2)*C2*0.0246615</f>
         <v>0.99856633035000009</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="3">
         <v>21.3</v>
@@ -1021,13 +1021,13 @@
         <v>2.77</v>
       </c>
       <c r="D3" s="4">
-        <f>SUM(B3-C3)*C3*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.2658279381500002</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3">
         <v>21.3</v>
@@ -1036,13 +1036,13 @@
         <v>2.77</v>
       </c>
       <c r="D4" s="4">
-        <f>SUM(B4-C4)*C4*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.2658279381500002</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3">
         <v>21.3</v>
@@ -1051,13 +1051,13 @@
         <v>3.73</v>
       </c>
       <c r="D5" s="4">
-        <f>SUM(B5-C5)*C5*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.6162185301500001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3">
         <v>21.3</v>
@@ -1066,13 +1066,13 @@
         <v>3.73</v>
       </c>
       <c r="D6" s="4">
-        <f>SUM(B6-C6)*C6*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.6162185301500001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3">
         <v>21.3</v>
@@ -1081,13 +1081,13 @@
         <v>4.78</v>
       </c>
       <c r="D7" s="4">
-        <f>SUM(B7-C7)*C7*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.9474101444000003</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3">
         <v>21.3</v>
@@ -1096,13 +1096,13 @@
         <v>7.47</v>
       </c>
       <c r="D8" s="4">
-        <f>SUM(B8-C8)*C8*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.5477820311500001</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3">
         <v>26.7</v>
@@ -1111,13 +1111,13 @@
         <v>2.11</v>
       </c>
       <c r="D9" s="4">
-        <f>SUM(B9-C9)*C9*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.2795594613499999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" s="3">
         <v>26.7</v>
@@ -1126,13 +1126,13 @@
         <v>2.87</v>
       </c>
       <c r="D10" s="4">
-        <f>SUM(B10-C10)*C10*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.68665177415</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" s="3">
         <v>26.7</v>
@@ -1141,13 +1141,13 @@
         <v>2.87</v>
       </c>
       <c r="D11" s="4">
-        <f>SUM(B11-C11)*C11*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>1.68665177415</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" s="3">
         <v>26.7</v>
@@ -1156,13 +1156,13 @@
         <v>3.91</v>
       </c>
       <c r="D12" s="4">
-        <f>SUM(B12-C12)*C12*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.1975591373500003</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="3">
         <v>26.7</v>
@@ -1171,13 +1171,13 @@
         <v>3.91</v>
       </c>
       <c r="D13" s="4">
-        <f>SUM(B13-C13)*C13*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.1975591373500003</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" s="3">
         <v>26.7</v>
@@ -1186,13 +1186,13 @@
         <v>5.56</v>
       </c>
       <c r="D14" s="4">
-        <f>SUM(B14-C14)*C14*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.8986732516</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" s="3">
         <v>26.7</v>
@@ -1201,13 +1201,13 @@
         <v>7.82</v>
       </c>
       <c r="D15" s="4">
-        <f>SUM(B15-C15)*C15*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.6410633184000001</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" s="3">
         <v>33.4</v>
@@ -1216,13 +1216,13 @@
         <v>2.77</v>
       </c>
       <c r="D16" s="4">
-        <f>SUM(B16-C16)*C16*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.09240743365</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17" s="3">
         <v>33.4</v>
@@ -1231,13 +1231,13 @@
         <v>3.38</v>
       </c>
       <c r="D17" s="4">
-        <f>SUM(B17-C17)*C17*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.5023432173999995</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>33.4</v>
@@ -1246,13 +1246,13 @@
         <v>3.38</v>
       </c>
       <c r="D18" s="4">
-        <f>SUM(B18-C18)*C18*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.5023432173999995</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19" s="3">
         <v>33.4</v>
@@ -1261,13 +1261,13 @@
         <v>4.55</v>
       </c>
       <c r="D19" s="4">
-        <f>SUM(B19-C19)*C19*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.2372534512499995</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B20" s="3">
         <v>33.4</v>
@@ -1276,13 +1276,13 @@
         <v>4.55</v>
       </c>
       <c r="D20" s="4">
-        <f>SUM(B20-C20)*C20*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.2372534512499995</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B21" s="3">
         <v>33.4</v>
@@ -1291,13 +1291,13 @@
         <v>6.35</v>
       </c>
       <c r="D21" s="4">
-        <f>SUM(B21-C21)*C21*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>4.2360442012499995</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B22" s="3">
         <v>33.4</v>
@@ -1306,13 +1306,13 @@
         <v>9.09</v>
       </c>
       <c r="D22" s="4">
-        <f>SUM(B22-C22)*C22*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>5.4496464808499994</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B23" s="3">
         <v>42.2</v>
@@ -1321,13 +1321,13 @@
         <v>2.77</v>
       </c>
       <c r="D23" s="4">
-        <f>SUM(B23-C23)*C23*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>2.6935561576500002</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B24" s="3">
         <v>42.2</v>
@@ -1336,13 +1336,13 @@
         <v>3.56</v>
       </c>
       <c r="D24" s="4">
-        <f>SUM(B24-C24)*C24*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.3923964816000001</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B25" s="3">
         <v>42.2</v>
@@ -1351,13 +1351,13 @@
         <v>3.56</v>
       </c>
       <c r="D25" s="4">
-        <f>SUM(B25-C25)*C25*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.3923964816000001</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B26" s="3">
         <v>42.2</v>
@@ -1366,13 +1366,13 @@
         <v>4.8499999999999996</v>
       </c>
       <c r="D26" s="4">
-        <f>SUM(B26-C26)*C26*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>4.4673690712499994</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B27" s="3">
         <v>42.2</v>
@@ -1381,13 +1381,13 @@
         <v>4.8499999999999996</v>
       </c>
       <c r="D27" s="4">
-        <f>SUM(B27-C27)*C27*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>4.4673690712499994</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B28" s="3">
         <v>42.2</v>
@@ -1396,13 +1396,13 @@
         <v>6.35</v>
       </c>
       <c r="D28" s="4">
-        <f>SUM(B28-C28)*C28*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>5.6141288212500005</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B29" s="3">
         <v>42.2</v>
@@ -1411,13 +1411,13 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="D29" s="4">
-        <f>SUM(B29-C29)*C29*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>7.774537875</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B30" s="3">
         <v>48.3</v>
@@ -1426,13 +1426,13 @@
         <v>2.77</v>
       </c>
       <c r="D30" s="4">
-        <f>SUM(B30-C30)*C30*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>3.1102615231499997</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31" s="3">
         <v>48.3</v>
@@ -1441,13 +1441,13 @@
         <v>3.68</v>
       </c>
       <c r="D31" s="4">
-        <f>SUM(B31-C31)*C31*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>4.0494577583999991</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32" s="3">
         <v>48.3</v>
@@ -1456,13 +1456,13 @@
         <v>3.68</v>
       </c>
       <c r="D32" s="4">
-        <f>SUM(B32-C32)*C32*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>4.0494577583999991</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B33" s="3">
         <v>48.3</v>
@@ -1471,13 +1471,13 @@
         <v>5.08</v>
       </c>
       <c r="D33" s="4">
-        <f>SUM(B33-C33)*C33*0.0246615</f>
+        <f t="shared" si="0"/>
         <v>5.4146197524000002</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B34" s="3">
         <v>48.3</v>
@@ -1486,13 +1486,13 @@
         <v>5.08</v>
       </c>
       <c r="D34" s="4">
-        <f>SUM(B34-C34)*C34*0.0246615</f>
+        <f t="shared" ref="D34:D65" si="1">SUM(B34-C34)*C34*0.0246615</f>
         <v>5.4146197524000002</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35" s="3">
         <v>48.3</v>
@@ -1501,13 +1501,13 @@
         <v>7.14</v>
       </c>
       <c r="D35" s="4">
-        <f>SUM(B35-C35)*C35*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>7.2475808075999986</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B36" s="3">
         <v>48.3</v>
@@ -1516,13 +1516,13 @@
         <v>10.16</v>
       </c>
       <c r="D36" s="4">
-        <f>SUM(B36-C36)*C36*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>9.5563904376000011</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B37" s="3">
         <v>60.3</v>
@@ -1531,13 +1531,13 @@
         <v>2.77</v>
       </c>
       <c r="D37" s="4">
-        <f>SUM(B37-C37)*C37*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>3.9300097831499996</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B38" s="3">
         <v>60.3</v>
@@ -1546,13 +1546,13 @@
         <v>3.91</v>
       </c>
       <c r="D38" s="4">
-        <f>SUM(B38-C38)*C38*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>5.4374883613499998</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B39" s="3">
         <v>60.3</v>
@@ -1561,13 +1561,13 @@
         <v>3.91</v>
       </c>
       <c r="D39" s="4">
-        <f>SUM(B39-C39)*C39*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>5.4374883613499998</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B40" s="3">
         <v>60.3</v>
@@ -1576,13 +1576,13 @@
         <v>5.54</v>
       </c>
       <c r="D40" s="4">
-        <f>SUM(B40-C40)*C40*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>7.4815691196000005</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B41" s="3">
         <v>60.3</v>
@@ -1591,13 +1591,13 @@
         <v>5.54</v>
       </c>
       <c r="D41" s="4">
-        <f>SUM(B41-C41)*C41*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>7.4815691196000005</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B42" s="3">
         <v>60.3</v>
@@ -1606,13 +1606,13 @@
         <v>8.74</v>
       </c>
       <c r="D42" s="4">
-        <f>SUM(B42-C42)*C42*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>11.1133202556</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B43" s="3">
         <v>60.3</v>
@@ -1621,13 +1621,13 @@
         <v>11.07</v>
       </c>
       <c r="D43" s="4">
-        <f>SUM(B43-C43)*C43*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>13.43992809015</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B44" s="3">
         <v>73</v>
@@ -1636,13 +1636,13 @@
         <v>3.05</v>
       </c>
       <c r="D44" s="4">
-        <f>SUM(B44-C44)*C44*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>5.2614693712499996</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B45" s="3">
         <v>73</v>
@@ -1651,13 +1651,13 @@
         <v>5.16</v>
       </c>
       <c r="D45" s="4">
-        <f>SUM(B45-C45)*C45*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>8.6328665856000004</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B46" s="3">
         <v>73</v>
@@ -1666,13 +1666,13 @@
         <v>5.16</v>
       </c>
       <c r="D46" s="4">
-        <f>SUM(B46-C46)*C46*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>8.6328665856000004</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B47" s="3">
         <v>73</v>
@@ -1681,13 +1681,13 @@
         <v>7.01</v>
       </c>
       <c r="D47" s="4">
-        <f>SUM(B47-C47)*C47*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>11.408160818849998</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B48" s="3">
         <v>73</v>
@@ -1696,13 +1696,13 @@
         <v>7.01</v>
       </c>
       <c r="D48" s="4">
-        <f>SUM(B48-C48)*C48*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>11.408160818849998</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B49" s="3">
         <v>73</v>
@@ -1711,13 +1711,13 @@
         <v>9.52</v>
       </c>
       <c r="D49" s="4">
-        <f>SUM(B49-C49)*C49*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>14.903674430400001</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B50" s="3">
         <v>73</v>
@@ -1726,13 +1726,13 @@
         <v>14.02</v>
       </c>
       <c r="D50" s="4">
-        <f>SUM(B50-C50)*C50*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>20.3925844854</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B51" s="3">
         <v>88.9</v>
@@ -1741,13 +1741,13 @@
         <v>3.05</v>
       </c>
       <c r="D51" s="4">
-        <f>SUM(B51-C51)*C51*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>6.4574288137500009</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B52" s="3">
         <v>88.9</v>
@@ -1756,13 +1756,13 @@
         <v>5.49</v>
       </c>
       <c r="D52" s="4">
-        <f>SUM(B52-C52)*C52*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>11.293016275350002</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B53" s="3">
         <v>88.9</v>
@@ -1771,13 +1771,13 @@
         <v>5.49</v>
       </c>
       <c r="D53" s="4">
-        <f>SUM(B53-C53)*C53*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>11.293016275350002</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B54" s="3">
         <v>88.9</v>
@@ -1786,13 +1786,13 @@
         <v>7.62</v>
       </c>
       <c r="D54" s="4">
-        <f>SUM(B54-C54)*C54*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>15.2741888064</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B55" s="3">
         <v>88.9</v>
@@ -1801,13 +1801,13 @@
         <v>7.62</v>
       </c>
       <c r="D55" s="4">
-        <f>SUM(B55-C55)*C55*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>15.2741888064</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B56" s="3">
         <v>88.9</v>
@@ -1816,13 +1816,13 @@
         <v>11.13</v>
       </c>
       <c r="D56" s="4">
-        <f>SUM(B56-C56)*C56*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>21.346503636150004</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B57" s="3">
         <v>88.9</v>
@@ -1831,13 +1831,13 @@
         <v>15.24</v>
       </c>
       <c r="D57" s="4">
-        <f>SUM(B57-C57)*C57*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>27.684467211600001</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B58" s="3">
         <v>114.3</v>
@@ -1846,13 +1846,13 @@
         <v>3.05</v>
       </c>
       <c r="D58" s="4">
-        <f>SUM(B58-C58)*C58*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>8.3679552187499997</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B59" s="3">
         <v>114.3</v>
@@ -1861,13 +1861,13 @@
         <v>6.02</v>
       </c>
       <c r="D59" s="4">
-        <f>SUM(B59-C59)*C59*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>16.075490264399999</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B60" s="3">
         <v>114.3</v>
@@ -1876,13 +1876,13 @@
         <v>6.02</v>
       </c>
       <c r="D60" s="4">
-        <f>SUM(B60-C60)*C60*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>16.075490264399999</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B61" s="3">
         <v>114.3</v>
@@ -1891,13 +1891,13 @@
         <v>8.56</v>
       </c>
       <c r="D61" s="4">
-        <f>SUM(B61-C61)*C61*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>22.321972005599999</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B62" s="3">
         <v>114.3</v>
@@ -1906,13 +1906,13 @@
         <v>8.56</v>
       </c>
       <c r="D62" s="4">
-        <f>SUM(B62-C62)*C62*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>22.321972005599999</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B63" s="3">
         <v>114.3</v>
@@ -1921,13 +1921,13 @@
         <v>11.13</v>
       </c>
       <c r="D63" s="4">
-        <f>SUM(B63-C63)*C63*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>28.318359009150001</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B64" s="3">
         <v>114.3</v>
@@ -1936,13 +1936,13 @@
         <v>13.49</v>
       </c>
       <c r="D64" s="4">
-        <f>SUM(B64-C64)*C64*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>33.537837244350001</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B65" s="3">
         <v>114.3</v>
@@ -1951,13 +1951,13 @@
         <v>17.12</v>
       </c>
       <c r="D65" s="4">
-        <f>SUM(B65-C65)*C65*0.0246615</f>
+        <f t="shared" si="1"/>
         <v>41.029870238400001</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B66" s="3">
         <v>141.30000000000001</v>
@@ -1966,13 +1966,13 @@
         <v>3.4</v>
       </c>
       <c r="D66" s="4">
-        <f>SUM(B66-C66)*C66*0.0246615</f>
+        <f t="shared" ref="D66:D97" si="2">SUM(B66-C66)*C66*0.0246615</f>
         <v>11.56279089</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B67" s="3">
         <v>141.30000000000001</v>
@@ -1981,13 +1981,13 @@
         <v>6.55</v>
       </c>
       <c r="D67" s="4">
-        <f>SUM(B67-C67)*C67*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>21.766548168749999</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B68" s="3">
         <v>141.30000000000001</v>
@@ -1996,13 +1996,13 @@
         <v>6.55</v>
       </c>
       <c r="D68" s="4">
-        <f>SUM(B68-C68)*C68*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>21.766548168749999</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B69" s="3">
         <v>141.30000000000001</v>
@@ -2011,13 +2011,13 @@
         <v>9.5299999999999994</v>
       </c>
       <c r="D69" s="4">
-        <f>SUM(B69-C69)*C69*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>30.969124998150001</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B70" s="3">
         <v>141.30000000000001</v>
@@ -2026,13 +2026,13 @@
         <v>9.5299999999999994</v>
       </c>
       <c r="D70" s="4">
-        <f>SUM(B70-C70)*C70*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>30.969124998150001</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B71" s="3">
         <v>141.30000000000001</v>
@@ -2041,13 +2041,13 @@
         <v>12.7</v>
       </c>
       <c r="D71" s="4">
-        <f>SUM(B71-C71)*C71*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>40.277655030000005</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B72" s="3">
         <v>141.30000000000001</v>
@@ -2056,13 +2056,13 @@
         <v>15.88</v>
       </c>
       <c r="D72" s="4">
-        <f>SUM(B72-C72)*C72*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>49.117559840400006</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B73" s="3">
         <v>141.30000000000001</v>
@@ -2071,13 +2071,13 @@
         <v>19.05</v>
       </c>
       <c r="D73" s="4">
-        <f>SUM(B73-C73)*C73*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>57.433242543750005</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B74" s="3">
         <v>168.3</v>
@@ -2086,13 +2086,13 @@
         <v>3.4</v>
       </c>
       <c r="D74" s="4">
-        <f>SUM(B74-C74)*C74*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>13.826716589999998</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B75" s="3">
         <v>168.3</v>
@@ -2101,13 +2101,13 @@
         <v>7.11</v>
       </c>
       <c r="D75" s="4">
-        <f>SUM(B75-C75)*C75*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>28.263580885349999</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B76" s="3">
         <v>168.3</v>
@@ -2116,13 +2116,13 @@
         <v>7.11</v>
       </c>
       <c r="D76" s="4">
-        <f>SUM(B76-C76)*C76*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>28.263580885349999</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B77" s="3">
         <v>168.3</v>
@@ -2131,13 +2131,13 @@
         <v>10.97</v>
       </c>
       <c r="D77" s="4">
-        <f>SUM(B77-C77)*C77*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>42.563531931150003</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B78" s="3">
         <v>168.3</v>
@@ -2146,13 +2146,13 @@
         <v>10.97</v>
       </c>
       <c r="D78" s="4">
-        <f>SUM(B78-C78)*C78*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>42.563531931150003</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B79" s="3">
         <v>168.3</v>
@@ -2161,13 +2161,13 @@
         <v>14.27</v>
       </c>
       <c r="D79" s="4">
-        <f>SUM(B79-C79)*C79*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>54.206176758150001</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B80" s="3">
         <v>168.3</v>
@@ -2176,13 +2176,13 @@
         <v>18.260000000000002</v>
       </c>
       <c r="D80" s="4">
-        <f>SUM(B80-C80)*C80*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>67.565861259600013</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B81" s="3">
         <v>168.3</v>
@@ -2191,13 +2191,13 @@
         <v>21.95</v>
       </c>
       <c r="D81" s="4">
-        <f>SUM(B81-C81)*C81*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>79.222171023750008</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B82" s="3">
         <v>219.1</v>
@@ -2206,13 +2206,13 @@
         <v>3.76</v>
       </c>
       <c r="D82" s="4">
-        <f>SUM(B82-C82)*C82*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>19.967883861600001</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B83" s="3">
         <v>219.1</v>
@@ -2221,13 +2221,13 @@
         <v>6.35</v>
       </c>
       <c r="D83" s="4">
-        <f>SUM(B83-C83)*C83*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>33.316761693749996</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B84" s="3">
         <v>219.1</v>
@@ -2236,13 +2236,13 @@
         <v>7.04</v>
       </c>
       <c r="D84" s="4">
-        <f>SUM(B84-C84)*C84*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>36.8172125376</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B85" s="3">
         <v>219.1</v>
@@ -2251,13 +2251,13 @@
         <v>8.18</v>
       </c>
       <c r="D85" s="4">
-        <f>SUM(B85-C85)*C85*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>42.549117284399998</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B86" s="3">
         <v>219.1</v>
@@ -2266,13 +2266,13 @@
         <v>8.18</v>
       </c>
       <c r="D86" s="4">
-        <f>SUM(B86-C86)*C86*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>42.549117284399998</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B87" s="3">
         <v>219.1</v>
@@ -2281,13 +2281,13 @@
         <v>10.31</v>
       </c>
       <c r="D87" s="4">
-        <f>SUM(B87-C87)*C87*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>53.086958971349993</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B88" s="3">
         <v>219.1</v>
@@ -2296,13 +2296,13 @@
         <v>12.7</v>
       </c>
       <c r="D88" s="4">
-        <f>SUM(B88-C88)*C88*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>64.644696719999999</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B89" s="3">
         <v>219.1</v>
@@ -2311,13 +2311,13 @@
         <v>12.7</v>
       </c>
       <c r="D89" s="4">
-        <f>SUM(B89-C89)*C89*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>64.644696719999999</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B90" s="3">
         <v>219.1</v>
@@ -2326,13 +2326,13 @@
         <v>15.09</v>
       </c>
       <c r="D90" s="4">
-        <f>SUM(B90-C90)*C90*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>75.920696560349995</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B91" s="3">
         <v>219.1</v>
@@ -2341,13 +2341,13 @@
         <v>18.260000000000002</v>
       </c>
       <c r="D91" s="4">
-        <f>SUM(B91-C91)*C91*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>90.442065951600014</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B92" s="3">
         <v>219.1</v>
@@ -2356,13 +2356,13 @@
         <v>20.62</v>
       </c>
       <c r="D92" s="4">
-        <f>SUM(B92-C92)*C92*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>100.9310754024</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B93" s="3">
         <v>219.1</v>
@@ -2371,13 +2371,13 @@
         <v>23.04</v>
       </c>
       <c r="D93" s="4">
-        <f>SUM(B93-C93)*C93*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>111.40148021759998</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B94" s="3">
         <v>219.1</v>
@@ -2386,13 +2386,13 @@
         <v>22.22</v>
       </c>
       <c r="D94" s="4">
-        <f>SUM(B94-C94)*C94*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>107.8860129864</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B95" s="3">
         <v>273</v>
@@ -2401,13 +2401,13 @@
         <v>4.1900000000000004</v>
       </c>
       <c r="D95" s="4">
-        <f>SUM(B95-C95)*C95*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>27.776590244850002</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B96" s="3">
         <v>273</v>
@@ -2416,13 +2416,13 @@
         <v>6.35</v>
       </c>
       <c r="D96" s="4">
-        <f>SUM(B96-C96)*C96*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>41.757529991249996</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B97" s="3">
         <v>273</v>
@@ -2431,13 +2431,13 @@
         <v>7.8</v>
       </c>
       <c r="D97" s="4">
-        <f>SUM(B97-C97)*C97*0.0246615</f>
+        <f t="shared" si="2"/>
         <v>51.013792439999996</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B98" s="3">
         <v>273</v>
@@ -2446,13 +2446,13 @@
         <v>9.27</v>
       </c>
       <c r="D98" s="4">
-        <f>SUM(B98-C98)*C98*0.0246615</f>
+        <f t="shared" ref="D98:D129" si="3">SUM(B98-C98)*C98*0.0246615</f>
         <v>60.291870451650006</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B99" s="3">
         <v>273</v>
@@ -2461,13 +2461,13 @@
         <v>9.27</v>
       </c>
       <c r="D99" s="4">
-        <f>SUM(B99-C99)*C99*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>60.291870451650006</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B100" s="3">
         <v>273</v>
@@ -2476,13 +2476,13 @@
         <v>12.7</v>
       </c>
       <c r="D100" s="4">
-        <f>SUM(B100-C100)*C100*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>81.526233314999999</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B101" s="3">
         <v>273</v>
@@ -2491,13 +2491,13 @@
         <v>12.7</v>
       </c>
       <c r="D101" s="4">
-        <f>SUM(B101-C101)*C101*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>81.526233314999999</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B102" s="3">
         <v>273</v>
@@ -2506,13 +2506,13 @@
         <v>15.09</v>
       </c>
       <c r="D102" s="4">
-        <f>SUM(B102-C102)*C102*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>95.979152246850006</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B103" s="3">
         <v>273</v>
@@ -2521,13 +2521,13 @@
         <v>18.260000000000002</v>
       </c>
       <c r="D103" s="4">
-        <f>SUM(B103-C103)*C103*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>114.71425951260001</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B104" s="3">
         <v>273</v>
@@ -2536,13 +2536,13 @@
         <v>21.44</v>
       </c>
       <c r="D104" s="4">
-        <f>SUM(B104-C104)*C104*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>133.01047839360001</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B105" s="3">
         <v>273</v>
@@ -2551,13 +2551,13 @@
         <v>25.4</v>
       </c>
       <c r="D105" s="4">
-        <f>SUM(B105-C105)*C105*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>155.09715995999997</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B106" s="3">
         <v>273</v>
@@ -2566,13 +2566,13 @@
         <v>28.58</v>
       </c>
       <c r="D106" s="4">
-        <f>SUM(B106-C106)*C106*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>172.27349026140001</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B107" s="3">
         <v>273</v>
@@ -2581,13 +2581,13 @@
         <v>25.4</v>
       </c>
       <c r="D107" s="4">
-        <f>SUM(B107-C107)*C107*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>155.09715995999997</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B108" s="3">
         <v>323.8</v>
@@ -2596,13 +2596,13 @@
         <v>4.57</v>
       </c>
       <c r="D108" s="4">
-        <f>SUM(B108-C108)*C108*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>35.978196247650004</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B109" s="3">
         <v>323.8</v>
@@ -2611,13 +2611,13 @@
         <v>6.35</v>
       </c>
       <c r="D109" s="4">
-        <f>SUM(B109-C109)*C109*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>49.712836661249995</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B110" s="3">
         <v>323.8</v>
@@ -2626,13 +2626,13 @@
         <v>8.3800000000000008</v>
       </c>
       <c r="D110" s="4">
-        <f>SUM(B110-C110)*C110*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>65.185760165400012</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B111" s="3">
         <v>323.8</v>
@@ -2641,13 +2641,13 @@
         <v>9.52</v>
       </c>
       <c r="D111" s="4">
-        <f>SUM(B111-C111)*C111*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>73.785866414400004</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B112" s="3">
         <v>323.8</v>
@@ -2656,13 +2656,13 @@
         <v>10.31</v>
       </c>
       <c r="D112" s="4">
-        <f>SUM(B112-C112)*C112*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>79.707987776850004</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B113" s="3">
         <v>323.8</v>
@@ -2671,13 +2671,13 @@
         <v>14.27</v>
       </c>
       <c r="D113" s="4">
-        <f>SUM(B113-C113)*C113*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>108.92967533565002</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B114" s="3">
         <v>323.8</v>
@@ -2686,13 +2686,13 @@
         <v>12.7</v>
       </c>
       <c r="D114" s="4">
-        <f>SUM(B114-C114)*C114*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>97.436846655000011</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B115" s="3">
         <v>323.8</v>
@@ -2701,13 +2701,13 @@
         <v>17.48</v>
       </c>
       <c r="D115" s="4">
-        <f>SUM(B115-C115)*C115*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>132.0493506864</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B116" s="3">
         <v>323.8</v>
@@ -2716,13 +2716,13 @@
         <v>21.44</v>
       </c>
       <c r="D116" s="4">
-        <f>SUM(B116-C116)*C116*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>159.8706004416</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B117" s="3">
         <v>323.8</v>
@@ -2731,13 +2731,13 @@
         <v>25.4</v>
       </c>
       <c r="D117" s="4">
-        <f>SUM(B117-C117)*C117*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>186.91838664000002</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B118" s="3">
         <v>323.8</v>
@@ -2746,13 +2746,13 @@
         <v>28.58</v>
       </c>
       <c r="D118" s="4">
-        <f>SUM(B118-C118)*C118*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>208.07863429739999</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B119" s="3">
         <v>323.8</v>
@@ -2761,13 +2761,13 @@
         <v>33.32</v>
       </c>
       <c r="D119" s="4">
-        <f>SUM(B119-C119)*C119*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>238.69356836640003</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B120" s="3">
         <v>323.8</v>
@@ -2776,13 +2776,13 @@
         <v>25.4</v>
       </c>
       <c r="D120" s="4">
-        <f>SUM(B120-C120)*C120*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>186.91838664000002</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B121" s="3">
         <v>355.6</v>
@@ -2791,13 +2791,13 @@
         <v>6.35</v>
       </c>
       <c r="D121" s="4">
-        <f>SUM(B121-C121)*C121*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>54.692733356249995</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B122" s="3">
         <v>355.6</v>
@@ -2806,13 +2806,13 @@
         <v>7.92</v>
       </c>
       <c r="D122" s="4">
-        <f>SUM(B122-C122)*C122*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>67.908537734399999</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B123" s="3">
         <v>355.6</v>
@@ -2821,13 +2821,13 @@
         <v>9.52</v>
       </c>
       <c r="D123" s="4">
-        <f>SUM(B123-C123)*C123*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>81.251790278400009</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B124" s="3">
         <v>355.6</v>
@@ -2836,13 +2836,13 @@
         <v>9.52</v>
       </c>
       <c r="D124" s="4">
-        <f>SUM(B124-C124)*C124*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>81.251790278400009</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B125" s="3">
         <v>355.6</v>
@@ -2851,13 +2851,13 @@
         <v>11.13</v>
       </c>
       <c r="D125" s="4">
-        <f>SUM(B125-C125)*C125*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>94.55098505265002</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B126" s="3">
         <v>355.6</v>
@@ -2866,13 +2866,13 @@
         <v>15.09</v>
       </c>
       <c r="D126" s="4">
-        <f>SUM(B126-C126)*C126*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>126.71808433785002</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B127" s="3">
         <v>355.6</v>
@@ -2881,13 +2881,13 @@
         <v>12.7</v>
       </c>
       <c r="D127" s="4">
-        <f>SUM(B127-C127)*C127*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>107.396640045</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B128" s="3">
         <v>355.6</v>
@@ -2896,13 +2896,13 @@
         <v>19.05</v>
       </c>
       <c r="D128" s="4">
-        <f>SUM(B128-C128)*C128*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>158.11172006625</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B129" s="3">
         <v>355.6</v>
@@ -2911,13 +2911,13 @@
         <v>23.83</v>
       </c>
       <c r="D129" s="4">
-        <f>SUM(B129-C129)*C129*0.0246615</f>
+        <f t="shared" si="3"/>
         <v>194.97576972465001</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B130" s="3">
         <v>355.6</v>
@@ -2926,13 +2926,13 @@
         <v>27.79</v>
       </c>
       <c r="D130" s="4">
-        <f>SUM(B130-C130)*C130*0.0246615</f>
+        <f t="shared" ref="D130:D161" si="4">SUM(B130-C130)*C130*0.0246615</f>
         <v>224.66231669384996</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B131" s="3">
         <v>355.6</v>
@@ -2941,13 +2941,13 @@
         <v>31.75</v>
       </c>
       <c r="D131" s="4">
-        <f>SUM(B131-C131)*C131*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>253.57540010625002</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B132" s="3">
         <v>355.6</v>
@@ -2956,13 +2956,13 @@
         <v>35.71</v>
       </c>
       <c r="D132" s="4">
-        <f>SUM(B132-C132)*C132*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>281.71501996185003</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B133" s="3">
         <v>406.4</v>
@@ -2971,13 +2971,13 @@
         <v>6.35</v>
       </c>
       <c r="D133" s="4">
-        <f>SUM(B133-C133)*C133*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>62.648040026249987</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B134" s="3">
         <v>406.4</v>
@@ -2986,13 +2986,13 @@
         <v>7.92</v>
       </c>
       <c r="D134" s="4">
-        <f>SUM(B134-C134)*C134*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>77.830746998399988</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B135" s="3">
         <v>406.4</v>
@@ -3001,13 +3001,13 @@
         <v>9.52</v>
       </c>
       <c r="D135" s="4">
-        <f>SUM(B135-C135)*C135*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>93.1784862624</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B136" s="3">
         <v>406.4</v>
@@ -3016,13 +3016,13 @@
         <v>9.52</v>
       </c>
       <c r="D136" s="4">
-        <f>SUM(B136-C136)*C136*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>93.1784862624</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B137" s="3">
         <v>406.4</v>
@@ -3031,13 +3031,13 @@
         <v>12.7</v>
       </c>
       <c r="D137" s="4">
-        <f>SUM(B137-C137)*C137*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>123.307253385</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B138" s="3">
         <v>406.4</v>
@@ -3046,13 +3046,13 @@
         <v>16.66</v>
       </c>
       <c r="D138" s="4">
-        <f>SUM(B138-C138)*C138*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>160.12880634659999</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B139" s="3">
         <v>406.4</v>
@@ -3061,13 +3061,13 @@
         <v>12.7</v>
       </c>
       <c r="D139" s="4">
-        <f>SUM(B139-C139)*C139*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>123.307253385</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B140" s="3">
         <v>406.4</v>
@@ -3076,13 +3076,13 @@
         <v>12.7</v>
       </c>
       <c r="D140" s="4">
-        <f>SUM(B140-C140)*C140*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>123.307253385</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B141" s="3">
         <v>406.4</v>
@@ -3091,13 +3091,13 @@
         <v>26.19</v>
       </c>
       <c r="D141" s="4">
-        <f>SUM(B141-C141)*C141*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>245.57181608385</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B142" s="3">
         <v>406.4</v>
@@ -3106,13 +3106,13 @@
         <v>30.96</v>
       </c>
       <c r="D142" s="4">
-        <f>SUM(B142-C142)*C142*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>286.65596381760002</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B143" s="3">
         <v>406.4</v>
@@ -3121,13 +3121,13 @@
         <v>36.53</v>
       </c>
       <c r="D143" s="4">
-        <f>SUM(B143-C143)*C143*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>333.21018515265001</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B144" s="3">
         <v>406.4</v>
@@ -3136,13 +3136,13 @@
         <v>40.49</v>
       </c>
       <c r="D144" s="4">
-        <f>SUM(B144-C144)*C144*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>365.37728443784994</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B145" s="3">
         <v>457</v>
@@ -3151,13 +3151,13 @@
         <v>6.35</v>
       </c>
       <c r="D145" s="4">
-        <f>SUM(B145-C145)*C145*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>70.572026591249994</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B146" s="3">
         <v>457</v>
@@ -3166,13 +3166,13 @@
         <v>7.92</v>
       </c>
       <c r="D146" s="4">
-        <f>SUM(B146-C146)*C146*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>87.713892446399996</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B147" s="3">
         <v>457</v>
@@ -3181,13 +3181,13 @@
         <v>11.13</v>
       </c>
       <c r="D147" s="4">
-        <f>SUM(B147-C147)*C147*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>122.38351004565001</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B148" s="3">
         <v>457</v>
@@ -3196,13 +3196,13 @@
         <v>9.52</v>
       </c>
       <c r="D148" s="4">
-        <f>SUM(B148-C148)*C148*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>105.05822675040001</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B149" s="3">
         <v>457</v>
@@ -3211,13 +3211,13 @@
         <v>14.27</v>
       </c>
       <c r="D149" s="4">
-        <f>SUM(B149-C149)*C149*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>155.80536672164999</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B150" s="3">
         <v>457</v>
@@ -3226,13 +3226,13 @@
         <v>19.05</v>
       </c>
       <c r="D150" s="4">
-        <f>SUM(B150-C150)*C150*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>205.74959977124999</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B151" s="3">
         <v>457</v>
@@ -3241,13 +3241,13 @@
         <v>12.7</v>
       </c>
       <c r="D151" s="4">
-        <f>SUM(B151-C151)*C151*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>139.15522651499998</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B152" s="3">
         <v>457</v>
@@ -3256,13 +3256,13 @@
         <v>23.83</v>
       </c>
       <c r="D152" s="4">
-        <f>SUM(B152-C152)*C152*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>254.56688118764998</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B153" s="3">
         <v>457</v>
@@ -3271,13 +3271,13 @@
         <v>29.36</v>
       </c>
       <c r="D153" s="4">
-        <f>SUM(B153-C153)*C153*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>309.63771972959995</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B154" s="3">
         <v>457</v>
@@ -3286,13 +3286,13 @@
         <v>34.92</v>
       </c>
       <c r="D154" s="4">
-        <f>SUM(B154-C154)*C154*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>363.48667712640002</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B155" s="3">
         <v>457</v>
@@ -3301,13 +3301,13 @@
         <v>39.67</v>
       </c>
       <c r="D155" s="4">
-        <f>SUM(B155-C155)*C155*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>408.28299714765001</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B156" s="3">
         <v>457</v>
@@ -3316,13 +3316,13 @@
         <v>45.24</v>
       </c>
       <c r="D156" s="4">
-        <f>SUM(B156-C156)*C156*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>459.39497441760005</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B157" s="3">
         <v>508</v>
@@ -3331,13 +3331,13 @@
         <v>6.35</v>
       </c>
       <c r="D157" s="4">
-        <f>SUM(B157-C157)*C157*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>78.558653366249985</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B158" s="3">
         <v>508</v>
@@ -3346,13 +3346,13 @@
         <v>9.52</v>
       </c>
       <c r="D158" s="4">
-        <f>SUM(B158-C158)*C158*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>117.0318782304</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B159" s="3">
         <v>508</v>
@@ -3361,13 +3361,13 @@
         <v>12.7</v>
       </c>
       <c r="D159" s="4">
-        <f>SUM(B159-C159)*C159*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>155.12848006499999</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B160" s="3">
         <v>508</v>
@@ -3376,13 +3376,13 @@
         <v>9.52</v>
       </c>
       <c r="D160" s="4">
-        <f>SUM(B160-C160)*C160*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>117.0318782304</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B161" s="3">
         <v>508</v>
@@ -3391,13 +3391,13 @@
         <v>15.09</v>
       </c>
       <c r="D161" s="4">
-        <f>SUM(B161-C161)*C161*0.0246615</f>
+        <f t="shared" si="4"/>
         <v>183.43253047185001</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B162" s="3">
         <v>508</v>
@@ -3412,7 +3412,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B163" s="3">
         <v>508</v>
@@ -3427,7 +3427,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B164" s="3">
         <v>508</v>
@@ -3442,7 +3442,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B165" s="3">
         <v>508</v>
@@ -3457,7 +3457,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B166" s="3">
         <v>508</v>
@@ -3472,7 +3472,7 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B167" s="3">
         <v>508</v>
@@ -3487,7 +3487,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B168" s="3">
         <v>508</v>
@@ -3502,7 +3502,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B169" s="3">
         <v>559</v>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B170" s="3">
         <v>559</v>
@@ -3532,7 +3532,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B171" s="3">
         <v>559</v>
@@ -3547,7 +3547,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B172" s="3">
         <v>559</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B173" s="3">
         <v>559</v>
@@ -3577,7 +3577,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B174" s="3">
         <v>559</v>
@@ -3592,7 +3592,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B175" s="3">
         <v>559</v>
@@ -3607,7 +3607,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B176" s="3">
         <v>559</v>
@@ -3622,7 +3622,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B177" s="3">
         <v>559</v>
@@ -3631,13 +3631,13 @@
         <v>34.92</v>
       </c>
       <c r="D177" s="4">
-        <f>SUM(B177-C177)*C177*0.0246615</f>
+        <f t="shared" ref="D177:D192" si="5">SUM(B177-C177)*C177*0.0246615</f>
         <v>451.32699428640007</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B178" s="3">
         <v>559</v>
@@ -3646,13 +3646,13 @@
         <v>41.28</v>
       </c>
       <c r="D178" s="4">
-        <f>SUM(B178-C178)*C178*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>527.05279347840008</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B179" s="3">
         <v>559</v>
@@ -3661,13 +3661,13 @@
         <v>47.62</v>
       </c>
       <c r="D179" s="4">
-        <f>SUM(B179-C179)*C179*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>600.55476656940004</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B180" s="3">
         <v>559</v>
@@ -3676,13 +3676,13 @@
         <v>53.98</v>
       </c>
       <c r="D180" s="4">
-        <f>SUM(B180-C180)*C180*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>672.29664840539999</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B181" s="3">
         <v>610</v>
@@ -3691,13 +3691,13 @@
         <v>6.35</v>
       </c>
       <c r="D181" s="4">
-        <f>SUM(B181-C181)*C181*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>94.531906916249994</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B182" s="3">
         <v>610</v>
@@ -3706,13 +3706,13 @@
         <v>9.52</v>
       </c>
       <c r="D182" s="4">
-        <f>SUM(B182-C182)*C182*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>140.9791811904</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B183" s="3">
         <v>610</v>
@@ -3721,13 +3721,13 @@
         <v>14.27</v>
       </c>
       <c r="D183" s="4">
-        <f>SUM(B183-C183)*C183*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>209.64906628665</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B184" s="3">
         <v>610</v>
@@ -3736,13 +3736,13 @@
         <v>9.5299999999999994</v>
       </c>
       <c r="D184" s="4">
-        <f>SUM(B184-C184)*C184*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>141.12491832465</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B185" s="3">
         <v>610</v>
@@ -3751,13 +3751,13 @@
         <v>17.48</v>
       </c>
       <c r="D185" s="4">
-        <f>SUM(B185-C185)*C185*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>255.42531101039998</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B186" s="3">
         <v>610</v>
@@ -3766,13 +3766,13 @@
         <v>24.61</v>
       </c>
       <c r="D186" s="4">
-        <f>SUM(B186-C186)*C186*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>355.28461488584998</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B187" s="3">
         <v>610</v>
@@ -3781,13 +3781,13 @@
         <v>12.7</v>
       </c>
       <c r="D187" s="4">
-        <f>SUM(B187-C187)*C187*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>187.07498716499998</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B188" s="3">
         <v>610</v>
@@ -3796,13 +3796,13 @@
         <v>30.96</v>
       </c>
       <c r="D188" s="4">
-        <f>SUM(B188-C188)*C188*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>442.10864396159997</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B189" s="3">
         <v>610</v>
@@ -3811,13 +3811,13 @@
         <v>38.89</v>
       </c>
       <c r="D189" s="4">
-        <f>SUM(B189-C189)*C189*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>547.74345411585</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B190" s="3">
         <v>610</v>
@@ -3826,13 +3826,13 @@
         <v>46.02</v>
       </c>
       <c r="D190" s="4">
-        <f>SUM(B190-C190)*C190*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>640.07343927540012</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B191" s="3">
         <v>610</v>
@@ -3841,13 +3841,13 @@
         <v>52.37</v>
       </c>
       <c r="D191" s="4">
-        <f>SUM(B191-C191)*C191*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>720.19183387064993</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B192" s="3">
         <v>610</v>
@@ -3856,7 +3856,7 @@
         <v>59.54</v>
       </c>
       <c r="D192" s="4">
-        <f>SUM(B192-C192)*C192*0.0246615</f>
+        <f t="shared" si="5"/>
         <v>808.26557952660005</v>
       </c>
     </row>

</xml_diff>